<commit_message>
Deploy data to app repo
</commit_message>
<xml_diff>
--- a/data/xlsx/Baernreither_Index_2023.xlsx
+++ b/data/xlsx/Baernreither_Index_2023.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10821"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11004"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/melaniedaubner/Documents/baernreither-data/data/xlsx/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D9329EBB-6E95-364E-88D3-BBF52B40CFFD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41FC107C-4E0D-3140-8E8F-06D2BBDDEFB1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="560" yWindow="6040" windowWidth="25600" windowHeight="14760" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3280" yWindow="1220" windowWidth="25600" windowHeight="14760" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="643" uniqueCount="343">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="646" uniqueCount="346">
   <si>
     <t>Hauptbegriff</t>
   </si>
@@ -1065,6 +1065,15 @@
   <si>
     <t>&lt;index&gt;&lt;term key="VereinigtesKoenigreich"&gt;  &lt;/term&gt;&lt;index&gt;&lt;term key="Sozialreform"/&gt;&lt;/index&gt;&lt;/index&gt;</t>
   </si>
+  <si>
+    <t>Annexion Bosniens und der Herzegowina</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Annexion Bosniens </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> &lt;index&gt;&lt;term key="AnnexionBosniens"&gt;&lt;/term&gt;&lt;/index&gt;</t>
+  </si>
 </sst>
 </file>
 
@@ -1487,7 +1496,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AC1064"/>
+  <dimension ref="A1:AC1065"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="14.5" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="34.5" style="4" customWidth="1"/>
@@ -1639,16 +1648,16 @@
       <c r="AC4" s="3"/>
     </row>
     <row r="5" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A5" s="8" t="s">
-        <v>6</v>
-      </c>
-      <c r="B5" s="3"/>
-      <c r="C5" s="8" t="s">
-        <v>6</v>
-      </c>
-      <c r="D5" s="3"/>
-      <c r="E5" s="3" t="s">
-        <v>7</v>
+      <c r="A5" s="35" t="s">
+        <v>343</v>
+      </c>
+      <c r="B5" s="28"/>
+      <c r="C5" s="35" t="s">
+        <v>344</v>
+      </c>
+      <c r="D5" s="28"/>
+      <c r="E5" s="28" t="s">
+        <v>345</v>
       </c>
       <c r="F5" s="3"/>
       <c r="G5" s="3"/>
@@ -1676,16 +1685,16 @@
       <c r="AC5" s="3"/>
     </row>
     <row r="6" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A6" s="1" t="s">
-        <v>8</v>
+      <c r="A6" s="8" t="s">
+        <v>6</v>
       </c>
       <c r="B6" s="3"/>
-      <c r="C6" s="1" t="s">
-        <v>8</v>
+      <c r="C6" s="8" t="s">
+        <v>6</v>
       </c>
       <c r="D6" s="3"/>
       <c r="E6" s="3" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="F6" s="3"/>
       <c r="G6" s="3"/>
@@ -1714,19 +1723,15 @@
     </row>
     <row r="7" spans="1:29" ht="15.75" customHeight="1">
       <c r="A7" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>11</v>
-      </c>
+        <v>8</v>
+      </c>
+      <c r="B7" s="3"/>
       <c r="C7" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="D7" s="3" t="s">
-        <v>11</v>
-      </c>
+        <v>8</v>
+      </c>
+      <c r="D7" s="3"/>
       <c r="E7" s="3" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="F7" s="3"/>
       <c r="G7" s="3"/>
@@ -1754,20 +1759,20 @@
       <c r="AC7" s="3"/>
     </row>
     <row r="8" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A8" s="9" t="s">
+      <c r="A8" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B8" s="10" t="s">
-        <v>13</v>
-      </c>
-      <c r="C8" s="9" t="s">
+      <c r="B8" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C8" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="D8" s="10" t="s">
-        <v>13</v>
-      </c>
-      <c r="E8" s="10" t="s">
-        <v>14</v>
+      <c r="D8" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>12</v>
       </c>
       <c r="F8" s="3"/>
       <c r="G8" s="3"/>
@@ -1795,20 +1800,20 @@
       <c r="AC8" s="3"/>
     </row>
     <row r="9" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A9" s="1" t="s">
+      <c r="A9" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="B9" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="C9" s="1" t="s">
+      <c r="B9" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="C9" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="D9" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="E9" s="3" t="s">
-        <v>16</v>
+      <c r="D9" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="E9" s="10" t="s">
+        <v>14</v>
       </c>
       <c r="F9" s="3"/>
       <c r="G9" s="3"/>
@@ -1836,20 +1841,20 @@
       <c r="AC9" s="3"/>
     </row>
     <row r="10" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A10" s="9" t="s">
+      <c r="A10" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B10" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="C10" s="9" t="s">
+      <c r="B10" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C10" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="D10" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="E10" s="11" t="s">
-        <v>18</v>
+      <c r="D10" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>16</v>
       </c>
       <c r="F10" s="3"/>
       <c r="G10" s="3"/>
@@ -1877,20 +1882,20 @@
       <c r="AC10" s="3"/>
     </row>
     <row r="11" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A11" s="1" t="s">
+      <c r="A11" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="B11" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="C11" s="1" t="s">
+      <c r="B11" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="C11" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="D11" s="3" t="s">
-        <v>20</v>
+      <c r="D11" s="10" t="s">
+        <v>17</v>
       </c>
       <c r="E11" s="11" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="F11" s="3"/>
       <c r="G11" s="3"/>
@@ -1919,19 +1924,19 @@
     </row>
     <row r="12" spans="1:29" ht="15.75" customHeight="1">
       <c r="A12" s="1" t="s">
-        <v>22</v>
+        <v>10</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>24</v>
+        <v>10</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="E12" s="11" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="F12" s="3"/>
       <c r="G12" s="3"/>
@@ -1963,16 +1968,16 @@
         <v>22</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="C13" s="1" t="s">
         <v>24</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="E13" s="11" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="F13" s="3"/>
       <c r="G13" s="3"/>
@@ -2004,16 +2009,16 @@
         <v>22</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C14" s="1" t="s">
         <v>24</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="E14" s="11" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="F14" s="3"/>
       <c r="G14" s="3"/>
@@ -2045,16 +2050,16 @@
         <v>22</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C15" s="1" t="s">
         <v>24</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="E15" s="11" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="F15" s="3"/>
       <c r="G15" s="3"/>
@@ -2082,16 +2087,20 @@
       <c r="AC15" s="3"/>
     </row>
     <row r="16" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A16" s="9" t="s">
-        <v>33</v>
-      </c>
-      <c r="B16" s="10"/>
-      <c r="C16" s="9" t="s">
-        <v>33</v>
-      </c>
-      <c r="D16" s="10"/>
+      <c r="A16" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="D16" s="3" t="s">
+        <v>31</v>
+      </c>
       <c r="E16" s="11" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="F16" s="3"/>
       <c r="G16" s="3"/>
@@ -2119,20 +2128,16 @@
       <c r="AC16" s="3"/>
     </row>
     <row r="17" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A17" s="12" t="s">
+      <c r="A17" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="B17" s="13" t="s">
-        <v>271</v>
-      </c>
-      <c r="C17" s="12" t="s">
+      <c r="B17" s="10"/>
+      <c r="C17" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="D17" s="13" t="s">
-        <v>271</v>
-      </c>
-      <c r="E17" s="13" t="s">
-        <v>272</v>
+      <c r="D17" s="10"/>
+      <c r="E17" s="11" t="s">
+        <v>34</v>
       </c>
       <c r="F17" s="3"/>
       <c r="G17" s="3"/>
@@ -2160,16 +2165,20 @@
       <c r="AC17" s="3"/>
     </row>
     <row r="18" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A18" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="B18" s="3"/>
-      <c r="C18" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="D18" s="3"/>
-      <c r="E18" s="11" t="s">
-        <v>37</v>
+      <c r="A18" s="12" t="s">
+        <v>33</v>
+      </c>
+      <c r="B18" s="13" t="s">
+        <v>271</v>
+      </c>
+      <c r="C18" s="12" t="s">
+        <v>33</v>
+      </c>
+      <c r="D18" s="13" t="s">
+        <v>271</v>
+      </c>
+      <c r="E18" s="13" t="s">
+        <v>272</v>
       </c>
       <c r="F18" s="3"/>
       <c r="G18" s="3"/>
@@ -2197,16 +2206,16 @@
       <c r="AC18" s="3"/>
     </row>
     <row r="19" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A19" s="9" t="s">
-        <v>38</v>
-      </c>
-      <c r="B19" s="10"/>
-      <c r="C19" s="9" t="s">
-        <v>39</v>
-      </c>
-      <c r="D19" s="10"/>
+      <c r="A19" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="B19" s="3"/>
+      <c r="C19" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="D19" s="3"/>
       <c r="E19" s="11" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="F19" s="3"/>
       <c r="G19" s="3"/>
@@ -2234,20 +2243,16 @@
       <c r="AC19" s="3"/>
     </row>
     <row r="20" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A20" s="35" t="s">
-        <v>41</v>
-      </c>
-      <c r="B20" s="28" t="s">
-        <v>286</v>
-      </c>
-      <c r="C20" s="35" t="s">
-        <v>43</v>
-      </c>
-      <c r="D20" s="28" t="s">
-        <v>287</v>
-      </c>
-      <c r="E20" s="28" t="s">
-        <v>338</v>
+      <c r="A20" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="B20" s="10"/>
+      <c r="C20" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="D20" s="10"/>
+      <c r="E20" s="11" t="s">
+        <v>40</v>
       </c>
       <c r="F20" s="3"/>
       <c r="G20" s="3"/>
@@ -2275,20 +2280,20 @@
       <c r="AC20" s="3"/>
     </row>
     <row r="21" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A21" s="1" t="s">
+      <c r="A21" s="35" t="s">
         <v>41</v>
       </c>
-      <c r="B21" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="C21" s="1" t="s">
+      <c r="B21" s="28" t="s">
+        <v>286</v>
+      </c>
+      <c r="C21" s="35" t="s">
         <v>43</v>
       </c>
-      <c r="D21" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="E21" s="3" t="s">
-        <v>45</v>
+      <c r="D21" s="28" t="s">
+        <v>287</v>
+      </c>
+      <c r="E21" s="28" t="s">
+        <v>338</v>
       </c>
       <c r="F21" s="3"/>
       <c r="G21" s="3"/>
@@ -2320,16 +2325,16 @@
         <v>41</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="C22" s="1" t="s">
         <v>43</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="E22" s="3" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="F22" s="3"/>
       <c r="G22" s="3"/>
@@ -2357,16 +2362,20 @@
       <c r="AC22" s="3"/>
     </row>
     <row r="23" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A23" s="9" t="s">
-        <v>48</v>
-      </c>
-      <c r="B23" s="10"/>
-      <c r="C23" s="9" t="s">
-        <v>48</v>
-      </c>
-      <c r="D23" s="10"/>
+      <c r="A23" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="B23" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="D23" s="3" t="s">
+        <v>46</v>
+      </c>
       <c r="E23" s="3" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="F23" s="3"/>
       <c r="G23" s="3"/>
@@ -2394,16 +2403,16 @@
       <c r="AC23" s="3"/>
     </row>
     <row r="24" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A24" s="12" t="s">
-        <v>273</v>
-      </c>
-      <c r="B24" s="13"/>
-      <c r="C24" s="12" t="s">
-        <v>273</v>
-      </c>
-      <c r="D24" s="13"/>
-      <c r="E24" s="13" t="s">
-        <v>274</v>
+      <c r="A24" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="B24" s="10"/>
+      <c r="C24" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="D24" s="10"/>
+      <c r="E24" s="3" t="s">
+        <v>49</v>
       </c>
       <c r="F24" s="3"/>
       <c r="G24" s="3"/>
@@ -2431,16 +2440,16 @@
       <c r="AC24" s="3"/>
     </row>
     <row r="25" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A25" s="9" t="s">
-        <v>50</v>
-      </c>
-      <c r="B25" s="10"/>
-      <c r="C25" s="9" t="s">
-        <v>50</v>
-      </c>
-      <c r="D25" s="10"/>
-      <c r="E25" s="3" t="s">
-        <v>51</v>
+      <c r="A25" s="12" t="s">
+        <v>273</v>
+      </c>
+      <c r="B25" s="13"/>
+      <c r="C25" s="12" t="s">
+        <v>273</v>
+      </c>
+      <c r="D25" s="13"/>
+      <c r="E25" s="13" t="s">
+        <v>274</v>
       </c>
       <c r="F25" s="3"/>
       <c r="G25" s="3"/>
@@ -2468,16 +2477,16 @@
       <c r="AC25" s="3"/>
     </row>
     <row r="26" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A26" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="B26" s="3"/>
-      <c r="C26" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="D26" s="3"/>
+      <c r="A26" s="9" t="s">
+        <v>50</v>
+      </c>
+      <c r="B26" s="10"/>
+      <c r="C26" s="9" t="s">
+        <v>50</v>
+      </c>
+      <c r="D26" s="10"/>
       <c r="E26" s="3" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="F26" s="3"/>
       <c r="G26" s="3"/>
@@ -2506,15 +2515,15 @@
     </row>
     <row r="27" spans="1:29" ht="15.75" customHeight="1">
       <c r="A27" s="1" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="B27" s="3"/>
       <c r="C27" s="1" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="D27" s="3"/>
       <c r="E27" s="3" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="F27" s="3"/>
       <c r="G27" s="3"/>
@@ -2542,16 +2551,16 @@
       <c r="AC27" s="3"/>
     </row>
     <row r="28" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A28" s="14" t="s">
-        <v>57</v>
-      </c>
-      <c r="B28" s="15"/>
-      <c r="C28" s="14" t="s">
-        <v>57</v>
-      </c>
-      <c r="D28" s="15"/>
+      <c r="A28" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="B28" s="3"/>
+      <c r="C28" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="D28" s="3"/>
       <c r="E28" s="3" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="F28" s="3"/>
       <c r="G28" s="3"/>
@@ -2579,16 +2588,16 @@
       <c r="AC28" s="3"/>
     </row>
     <row r="29" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A29" s="33" t="s">
-        <v>326</v>
-      </c>
-      <c r="B29" s="34"/>
-      <c r="C29" s="33" t="s">
-        <v>327</v>
-      </c>
-      <c r="D29" s="34"/>
-      <c r="E29" s="28" t="s">
-        <v>328</v>
+      <c r="A29" s="14" t="s">
+        <v>57</v>
+      </c>
+      <c r="B29" s="15"/>
+      <c r="C29" s="14" t="s">
+        <v>57</v>
+      </c>
+      <c r="D29" s="15"/>
+      <c r="E29" s="3" t="s">
+        <v>58</v>
       </c>
       <c r="F29" s="3"/>
       <c r="G29" s="3"/>
@@ -2619,17 +2628,13 @@
       <c r="A30" s="33" t="s">
         <v>326</v>
       </c>
-      <c r="B30" s="34" t="s">
-        <v>329</v>
-      </c>
+      <c r="B30" s="34"/>
       <c r="C30" s="33" t="s">
         <v>327</v>
       </c>
-      <c r="D30" s="34" t="s">
-        <v>330</v>
-      </c>
+      <c r="D30" s="34"/>
       <c r="E30" s="28" t="s">
-        <v>331</v>
+        <v>328</v>
       </c>
       <c r="F30" s="3"/>
       <c r="G30" s="3"/>
@@ -2657,16 +2662,20 @@
       <c r="AC30" s="3"/>
     </row>
     <row r="31" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A31" s="16" t="s">
-        <v>275</v>
-      </c>
-      <c r="B31" s="17"/>
-      <c r="C31" s="16" t="s">
-        <v>275</v>
-      </c>
-      <c r="D31" s="17"/>
-      <c r="E31" s="13" t="s">
-        <v>276</v>
+      <c r="A31" s="33" t="s">
+        <v>326</v>
+      </c>
+      <c r="B31" s="34" t="s">
+        <v>329</v>
+      </c>
+      <c r="C31" s="33" t="s">
+        <v>327</v>
+      </c>
+      <c r="D31" s="34" t="s">
+        <v>330</v>
+      </c>
+      <c r="E31" s="28" t="s">
+        <v>331</v>
       </c>
       <c r="F31" s="3"/>
       <c r="G31" s="3"/>
@@ -2694,20 +2703,16 @@
       <c r="AC31" s="3"/>
     </row>
     <row r="32" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A32" s="35" t="s">
-        <v>332</v>
-      </c>
-      <c r="B32" s="28" t="s">
-        <v>339</v>
-      </c>
-      <c r="C32" s="35" t="s">
-        <v>332</v>
-      </c>
-      <c r="D32" s="28" t="s">
-        <v>339</v>
-      </c>
-      <c r="E32" s="28" t="s">
-        <v>340</v>
+      <c r="A32" s="16" t="s">
+        <v>275</v>
+      </c>
+      <c r="B32" s="17"/>
+      <c r="C32" s="16" t="s">
+        <v>275</v>
+      </c>
+      <c r="D32" s="17"/>
+      <c r="E32" s="13" t="s">
+        <v>276</v>
       </c>
       <c r="F32" s="3"/>
       <c r="G32" s="3"/>
@@ -2739,16 +2744,16 @@
         <v>332</v>
       </c>
       <c r="B33" s="28" t="s">
-        <v>333</v>
+        <v>339</v>
       </c>
       <c r="C33" s="35" t="s">
         <v>332</v>
       </c>
       <c r="D33" s="28" t="s">
-        <v>334</v>
+        <v>339</v>
       </c>
       <c r="E33" s="28" t="s">
-        <v>335</v>
+        <v>340</v>
       </c>
       <c r="F33" s="3"/>
       <c r="G33" s="3"/>
@@ -2780,16 +2785,16 @@
         <v>332</v>
       </c>
       <c r="B34" s="28" t="s">
-        <v>46</v>
+        <v>333</v>
       </c>
       <c r="C34" s="35" t="s">
         <v>332</v>
       </c>
       <c r="D34" s="28" t="s">
-        <v>46</v>
+        <v>334</v>
       </c>
       <c r="E34" s="28" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="F34" s="3"/>
       <c r="G34" s="3"/>
@@ -2821,16 +2826,16 @@
         <v>332</v>
       </c>
       <c r="B35" s="28" t="s">
-        <v>77</v>
+        <v>46</v>
       </c>
       <c r="C35" s="35" t="s">
         <v>332</v>
       </c>
       <c r="D35" s="28" t="s">
-        <v>77</v>
+        <v>46</v>
       </c>
       <c r="E35" s="28" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="F35" s="3"/>
       <c r="G35" s="3"/>
@@ -2858,20 +2863,20 @@
       <c r="AC35" s="3"/>
     </row>
     <row r="36" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A36" s="18" t="s">
-        <v>59</v>
-      </c>
-      <c r="B36" s="18" t="s">
-        <v>60</v>
-      </c>
-      <c r="C36" s="18" t="s">
-        <v>61</v>
-      </c>
-      <c r="D36" s="18" t="s">
-        <v>60</v>
-      </c>
-      <c r="E36" s="3" t="s">
-        <v>62</v>
+      <c r="A36" s="35" t="s">
+        <v>332</v>
+      </c>
+      <c r="B36" s="28" t="s">
+        <v>77</v>
+      </c>
+      <c r="C36" s="35" t="s">
+        <v>332</v>
+      </c>
+      <c r="D36" s="28" t="s">
+        <v>77</v>
+      </c>
+      <c r="E36" s="28" t="s">
+        <v>337</v>
       </c>
       <c r="F36" s="3"/>
       <c r="G36" s="3"/>
@@ -2899,20 +2904,20 @@
       <c r="AC36" s="3"/>
     </row>
     <row r="37" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A37" s="19" t="s">
+      <c r="A37" s="18" t="s">
         <v>59</v>
       </c>
-      <c r="B37" s="19" t="s">
-        <v>277</v>
-      </c>
-      <c r="C37" s="19" t="s">
+      <c r="B37" s="18" t="s">
+        <v>60</v>
+      </c>
+      <c r="C37" s="18" t="s">
         <v>61</v>
       </c>
-      <c r="D37" s="19" t="s">
-        <v>277</v>
+      <c r="D37" s="18" t="s">
+        <v>60</v>
       </c>
       <c r="E37" s="3" t="s">
-        <v>278</v>
+        <v>62</v>
       </c>
       <c r="F37" s="3"/>
       <c r="G37" s="3"/>
@@ -2944,16 +2949,16 @@
         <v>59</v>
       </c>
       <c r="B38" s="19" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="C38" s="19" t="s">
         <v>61</v>
       </c>
       <c r="D38" s="19" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="E38" s="3" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="F38" s="3"/>
       <c r="G38" s="3"/>
@@ -2981,20 +2986,20 @@
       <c r="AC38" s="3"/>
     </row>
     <row r="39" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A39" s="20" t="s">
-        <v>63</v>
-      </c>
-      <c r="B39" s="3" t="s">
-        <v>64</v>
-      </c>
-      <c r="C39" s="20" t="s">
-        <v>269</v>
-      </c>
-      <c r="D39" s="3" t="s">
-        <v>65</v>
+      <c r="A39" s="19" t="s">
+        <v>59</v>
+      </c>
+      <c r="B39" s="19" t="s">
+        <v>279</v>
+      </c>
+      <c r="C39" s="19" t="s">
+        <v>61</v>
+      </c>
+      <c r="D39" s="19" t="s">
+        <v>279</v>
       </c>
       <c r="E39" s="3" t="s">
-        <v>66</v>
+        <v>280</v>
       </c>
       <c r="F39" s="3"/>
       <c r="G39" s="3"/>
@@ -3022,20 +3027,20 @@
       <c r="AC39" s="3"/>
     </row>
     <row r="40" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A40" s="1" t="s">
-        <v>67</v>
+      <c r="A40" s="20" t="s">
+        <v>63</v>
       </c>
       <c r="B40" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="C40" s="1" t="s">
-        <v>67</v>
+        <v>64</v>
+      </c>
+      <c r="C40" s="20" t="s">
+        <v>269</v>
       </c>
       <c r="D40" s="3" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="E40" s="3" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="F40" s="3"/>
       <c r="G40" s="3"/>
@@ -3064,15 +3069,19 @@
     </row>
     <row r="41" spans="1:29" ht="15.75" customHeight="1">
       <c r="A41" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="B41" s="3"/>
+        <v>67</v>
+      </c>
+      <c r="B41" s="3" t="s">
+        <v>68</v>
+      </c>
       <c r="C41" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="D41" s="3"/>
+        <v>67</v>
+      </c>
+      <c r="D41" s="3" t="s">
+        <v>68</v>
+      </c>
       <c r="E41" s="3" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="F41" s="3"/>
       <c r="G41" s="3"/>
@@ -3101,15 +3110,15 @@
     </row>
     <row r="42" spans="1:29" ht="15.75" customHeight="1">
       <c r="A42" s="1" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="B42" s="3"/>
       <c r="C42" s="1" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="D42" s="3"/>
       <c r="E42" s="3" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="F42" s="3"/>
       <c r="G42" s="3"/>
@@ -3138,15 +3147,15 @@
     </row>
     <row r="43" spans="1:29" ht="15.75" customHeight="1">
       <c r="A43" s="1" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="B43" s="3"/>
       <c r="C43" s="1" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="D43" s="3"/>
       <c r="E43" s="3" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="F43" s="3"/>
       <c r="G43" s="3"/>
@@ -3177,17 +3186,13 @@
       <c r="A44" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="B44" s="3" t="s">
-        <v>77</v>
-      </c>
+      <c r="B44" s="3"/>
       <c r="C44" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="D44" s="3" t="s">
-        <v>77</v>
-      </c>
+      <c r="D44" s="3"/>
       <c r="E44" s="3" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="F44" s="3"/>
       <c r="G44" s="3"/>
@@ -3215,20 +3220,20 @@
       <c r="AC44" s="3"/>
     </row>
     <row r="45" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A45" s="9" t="s">
+      <c r="A45" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="B45" s="10" t="s">
-        <v>79</v>
-      </c>
-      <c r="C45" s="9" t="s">
+      <c r="B45" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="C45" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="D45" s="10" t="s">
-        <v>80</v>
-      </c>
-      <c r="E45" s="11" t="s">
-        <v>81</v>
+      <c r="D45" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="E45" s="3" t="s">
+        <v>78</v>
       </c>
       <c r="F45" s="3"/>
       <c r="G45" s="3"/>
@@ -3260,16 +3265,16 @@
         <v>74</v>
       </c>
       <c r="B46" s="10" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="C46" s="9" t="s">
         <v>75</v>
       </c>
       <c r="D46" s="10" t="s">
-        <v>83</v>
-      </c>
-      <c r="E46" s="3" t="s">
-        <v>84</v>
+        <v>80</v>
+      </c>
+      <c r="E46" s="11" t="s">
+        <v>81</v>
       </c>
       <c r="F46" s="3"/>
       <c r="G46" s="3"/>
@@ -3297,20 +3302,20 @@
       <c r="AC46" s="3"/>
     </row>
     <row r="47" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A47" s="12" t="s">
+      <c r="A47" s="9" t="s">
         <v>74</v>
       </c>
-      <c r="B47" s="13" t="s">
-        <v>281</v>
-      </c>
-      <c r="C47" s="12" t="s">
+      <c r="B47" s="10" t="s">
+        <v>82</v>
+      </c>
+      <c r="C47" s="9" t="s">
         <v>75</v>
       </c>
-      <c r="D47" s="13" t="s">
-        <v>95</v>
-      </c>
-      <c r="E47" s="13" t="s">
-        <v>282</v>
+      <c r="D47" s="10" t="s">
+        <v>83</v>
+      </c>
+      <c r="E47" s="3" t="s">
+        <v>84</v>
       </c>
       <c r="F47" s="3"/>
       <c r="G47" s="3"/>
@@ -3338,20 +3343,20 @@
       <c r="AC47" s="3"/>
     </row>
     <row r="48" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A48" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="B48" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="C48" s="1" t="s">
-        <v>86</v>
-      </c>
-      <c r="D48" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="E48" s="21" t="s">
-        <v>87</v>
+      <c r="A48" s="12" t="s">
+        <v>74</v>
+      </c>
+      <c r="B48" s="13" t="s">
+        <v>281</v>
+      </c>
+      <c r="C48" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="D48" s="13" t="s">
+        <v>95</v>
+      </c>
+      <c r="E48" s="13" t="s">
+        <v>282</v>
       </c>
       <c r="F48" s="3"/>
       <c r="G48" s="3"/>
@@ -3379,20 +3384,20 @@
       <c r="AC48" s="3"/>
     </row>
     <row r="49" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A49" s="9" t="s">
+      <c r="A49" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="B49" s="10" t="s">
-        <v>88</v>
+      <c r="B49" s="3" t="s">
+        <v>57</v>
       </c>
       <c r="C49" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="D49" s="10" t="s">
-        <v>88</v>
+      <c r="D49" s="3" t="s">
+        <v>57</v>
       </c>
       <c r="E49" s="21" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="F49" s="3"/>
       <c r="G49" s="3"/>
@@ -3420,20 +3425,20 @@
       <c r="AC49" s="3"/>
     </row>
     <row r="50" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A50" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="B50" s="3" t="s">
-        <v>83</v>
+      <c r="A50" s="9" t="s">
+        <v>85</v>
+      </c>
+      <c r="B50" s="10" t="s">
+        <v>88</v>
       </c>
       <c r="C50" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="D50" s="3" t="s">
-        <v>83</v>
-      </c>
-      <c r="E50" s="22" t="s">
-        <v>92</v>
+        <v>86</v>
+      </c>
+      <c r="D50" s="10" t="s">
+        <v>88</v>
+      </c>
+      <c r="E50" s="21" t="s">
+        <v>89</v>
       </c>
       <c r="F50" s="3"/>
       <c r="G50" s="3"/>
@@ -3461,20 +3466,20 @@
       <c r="AC50" s="3"/>
     </row>
     <row r="51" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A51" s="12" t="s">
+      <c r="A51" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="B51" s="13" t="s">
-        <v>283</v>
-      </c>
-      <c r="C51" s="12" t="s">
+      <c r="B51" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="C51" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="D51" s="13" t="s">
-        <v>284</v>
+      <c r="D51" s="3" t="s">
+        <v>83</v>
       </c>
       <c r="E51" s="22" t="s">
-        <v>285</v>
+        <v>92</v>
       </c>
       <c r="F51" s="3"/>
       <c r="G51" s="3"/>
@@ -3502,20 +3507,20 @@
       <c r="AC51" s="3"/>
     </row>
     <row r="52" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A52" s="9" t="s">
+      <c r="A52" s="12" t="s">
         <v>90</v>
       </c>
-      <c r="B52" s="10" t="s">
-        <v>93</v>
-      </c>
-      <c r="C52" s="1" t="s">
+      <c r="B52" s="13" t="s">
+        <v>283</v>
+      </c>
+      <c r="C52" s="12" t="s">
         <v>91</v>
       </c>
-      <c r="D52" s="10" t="s">
-        <v>93</v>
+      <c r="D52" s="13" t="s">
+        <v>284</v>
       </c>
       <c r="E52" s="22" t="s">
-        <v>94</v>
+        <v>285</v>
       </c>
       <c r="F52" s="3"/>
       <c r="G52" s="3"/>
@@ -3547,16 +3552,16 @@
         <v>90</v>
       </c>
       <c r="B53" s="10" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="C53" s="1" t="s">
         <v>91</v>
       </c>
       <c r="D53" s="10" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="E53" s="22" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="F53" s="3"/>
       <c r="G53" s="3"/>
@@ -3584,20 +3589,20 @@
       <c r="AC53" s="3"/>
     </row>
     <row r="54" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A54" s="1" t="s">
+      <c r="A54" s="9" t="s">
         <v>90</v>
       </c>
-      <c r="B54" s="3" t="s">
-        <v>33</v>
+      <c r="B54" s="10" t="s">
+        <v>95</v>
       </c>
       <c r="C54" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="D54" s="3" t="s">
-        <v>33</v>
+      <c r="D54" s="10" t="s">
+        <v>95</v>
       </c>
       <c r="E54" s="22" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="F54" s="3"/>
       <c r="G54" s="3"/>
@@ -3625,20 +3630,20 @@
       <c r="AC54" s="3"/>
     </row>
     <row r="55" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A55" s="12" t="s">
+      <c r="A55" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="B55" s="13" t="s">
-        <v>286</v>
-      </c>
-      <c r="C55" s="12" t="s">
+      <c r="B55" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="C55" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="D55" s="13" t="s">
-        <v>287</v>
-      </c>
-      <c r="E55" s="13" t="s">
-        <v>288</v>
+      <c r="D55" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="E55" s="22" t="s">
+        <v>97</v>
       </c>
       <c r="F55" s="3"/>
       <c r="G55" s="3"/>
@@ -3666,20 +3671,20 @@
       <c r="AC55" s="3"/>
     </row>
     <row r="56" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A56" s="1" t="s">
+      <c r="A56" s="12" t="s">
         <v>90</v>
       </c>
-      <c r="B56" s="3" t="s">
-        <v>98</v>
-      </c>
-      <c r="C56" s="1" t="s">
+      <c r="B56" s="13" t="s">
+        <v>286</v>
+      </c>
+      <c r="C56" s="12" t="s">
         <v>91</v>
       </c>
-      <c r="D56" s="3" t="s">
-        <v>99</v>
-      </c>
-      <c r="E56" s="22" t="s">
-        <v>100</v>
+      <c r="D56" s="13" t="s">
+        <v>287</v>
+      </c>
+      <c r="E56" s="13" t="s">
+        <v>288</v>
       </c>
       <c r="F56" s="3"/>
       <c r="G56" s="3"/>
@@ -3707,20 +3712,20 @@
       <c r="AC56" s="3"/>
     </row>
     <row r="57" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A57" s="9" t="s">
+      <c r="A57" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="B57" s="10" t="s">
-        <v>101</v>
+      <c r="B57" s="3" t="s">
+        <v>98</v>
       </c>
       <c r="C57" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="D57" s="10" t="s">
-        <v>102</v>
+      <c r="D57" s="3" t="s">
+        <v>99</v>
       </c>
       <c r="E57" s="22" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="F57" s="3"/>
       <c r="G57" s="3"/>
@@ -3752,16 +3757,16 @@
         <v>90</v>
       </c>
       <c r="B58" s="10" t="s">
-        <v>57</v>
+        <v>101</v>
       </c>
       <c r="C58" s="1" t="s">
         <v>91</v>
       </c>
       <c r="D58" s="10" t="s">
-        <v>57</v>
+        <v>102</v>
       </c>
       <c r="E58" s="22" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="F58" s="3"/>
       <c r="G58" s="3"/>
@@ -3789,20 +3794,20 @@
       <c r="AC58" s="3"/>
     </row>
     <row r="59" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A59" s="1" t="s">
+      <c r="A59" s="9" t="s">
         <v>90</v>
       </c>
-      <c r="B59" s="3" t="s">
-        <v>105</v>
+      <c r="B59" s="10" t="s">
+        <v>57</v>
       </c>
       <c r="C59" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="D59" s="3" t="s">
-        <v>105</v>
-      </c>
-      <c r="E59" s="3" t="s">
-        <v>106</v>
+      <c r="D59" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="E59" s="22" t="s">
+        <v>104</v>
       </c>
       <c r="F59" s="3"/>
       <c r="G59" s="3"/>
@@ -3834,16 +3839,16 @@
         <v>90</v>
       </c>
       <c r="B60" s="3" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C60" s="1" t="s">
         <v>91</v>
       </c>
       <c r="D60" s="3" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="E60" s="3" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="F60" s="3"/>
       <c r="G60" s="3"/>
@@ -3875,16 +3880,16 @@
         <v>90</v>
       </c>
       <c r="B61" s="3" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="C61" s="1" t="s">
         <v>91</v>
       </c>
       <c r="D61" s="3" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="E61" s="3" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="F61" s="3"/>
       <c r="G61" s="3"/>
@@ -3916,16 +3921,16 @@
         <v>90</v>
       </c>
       <c r="B62" s="3" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="C62" s="1" t="s">
         <v>91</v>
       </c>
       <c r="D62" s="3" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="E62" s="3" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="F62" s="3"/>
       <c r="G62" s="3"/>
@@ -3957,16 +3962,16 @@
         <v>90</v>
       </c>
       <c r="B63" s="3" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="C63" s="1" t="s">
         <v>91</v>
       </c>
       <c r="D63" s="3" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="E63" s="3" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="F63" s="3"/>
       <c r="G63" s="3"/>
@@ -3998,16 +4003,16 @@
         <v>90</v>
       </c>
       <c r="B64" s="3" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="C64" s="1" t="s">
         <v>91</v>
       </c>
       <c r="D64" s="3" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="E64" s="3" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="F64" s="3"/>
       <c r="G64" s="3"/>
@@ -4039,16 +4044,16 @@
         <v>90</v>
       </c>
       <c r="B65" s="3" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="C65" s="1" t="s">
         <v>91</v>
       </c>
       <c r="D65" s="3" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="E65" s="3" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="F65" s="3"/>
       <c r="G65" s="3"/>
@@ -4076,20 +4081,20 @@
       <c r="AC65" s="3"/>
     </row>
     <row r="66" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A66" s="12" t="s">
+      <c r="A66" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="B66" s="13" t="s">
-        <v>289</v>
-      </c>
-      <c r="C66" s="12" t="s">
+      <c r="B66" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="C66" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="D66" s="13" t="s">
-        <v>289</v>
-      </c>
-      <c r="E66" s="22" t="s">
-        <v>290</v>
+      <c r="D66" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="E66" s="3" t="s">
+        <v>121</v>
       </c>
       <c r="F66" s="3"/>
       <c r="G66" s="3"/>
@@ -4117,20 +4122,20 @@
       <c r="AC66" s="3"/>
     </row>
     <row r="67" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A67" s="1" t="s">
+      <c r="A67" s="12" t="s">
         <v>90</v>
       </c>
-      <c r="B67" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="C67" s="1" t="s">
+      <c r="B67" s="13" t="s">
+        <v>289</v>
+      </c>
+      <c r="C67" s="12" t="s">
         <v>91</v>
       </c>
-      <c r="D67" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="E67" s="3" t="s">
-        <v>122</v>
+      <c r="D67" s="13" t="s">
+        <v>289</v>
+      </c>
+      <c r="E67" s="22" t="s">
+        <v>290</v>
       </c>
       <c r="F67" s="3"/>
       <c r="G67" s="3"/>
@@ -4162,16 +4167,16 @@
         <v>90</v>
       </c>
       <c r="B68" s="3" t="s">
-        <v>123</v>
+        <v>46</v>
       </c>
       <c r="C68" s="1" t="s">
         <v>91</v>
       </c>
       <c r="D68" s="3" t="s">
-        <v>123</v>
+        <v>46</v>
       </c>
       <c r="E68" s="3" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="F68" s="3"/>
       <c r="G68" s="3"/>
@@ -4199,16 +4204,20 @@
       <c r="AC68" s="3"/>
     </row>
     <row r="69" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A69" s="12" t="s">
-        <v>291</v>
-      </c>
-      <c r="B69" s="13"/>
-      <c r="C69" s="12" t="s">
-        <v>291</v>
-      </c>
-      <c r="D69" s="13"/>
-      <c r="E69" s="13" t="s">
-        <v>292</v>
+      <c r="A69" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="B69" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="C69" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="D69" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="E69" s="3" t="s">
+        <v>124</v>
       </c>
       <c r="F69" s="3"/>
       <c r="G69" s="3"/>
@@ -4236,16 +4245,16 @@
       <c r="AC69" s="3"/>
     </row>
     <row r="70" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A70" s="1" t="s">
-        <v>125</v>
-      </c>
-      <c r="B70" s="3"/>
-      <c r="C70" s="1" t="s">
-        <v>125</v>
-      </c>
-      <c r="D70" s="3"/>
-      <c r="E70" s="3" t="s">
-        <v>126</v>
+      <c r="A70" s="12" t="s">
+        <v>291</v>
+      </c>
+      <c r="B70" s="13"/>
+      <c r="C70" s="12" t="s">
+        <v>291</v>
+      </c>
+      <c r="D70" s="13"/>
+      <c r="E70" s="13" t="s">
+        <v>292</v>
       </c>
       <c r="F70" s="3"/>
       <c r="G70" s="3"/>
@@ -4273,16 +4282,16 @@
       <c r="AC70" s="3"/>
     </row>
     <row r="71" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A71" s="12" t="s">
-        <v>293</v>
-      </c>
-      <c r="B71" s="13"/>
-      <c r="C71" s="12" t="s">
-        <v>293</v>
-      </c>
-      <c r="D71" s="13"/>
-      <c r="E71" s="13" t="s">
-        <v>294</v>
+      <c r="A71" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="B71" s="3"/>
+      <c r="C71" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="D71" s="3"/>
+      <c r="E71" s="3" t="s">
+        <v>126</v>
       </c>
       <c r="F71" s="3"/>
       <c r="G71" s="3"/>
@@ -4310,16 +4319,16 @@
       <c r="AC71" s="3"/>
     </row>
     <row r="72" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A72" s="1" t="s">
-        <v>127</v>
-      </c>
-      <c r="B72" s="3"/>
-      <c r="C72" s="1" t="s">
-        <v>127</v>
-      </c>
-      <c r="D72" s="3"/>
-      <c r="E72" s="3" t="s">
-        <v>128</v>
+      <c r="A72" s="12" t="s">
+        <v>293</v>
+      </c>
+      <c r="B72" s="13"/>
+      <c r="C72" s="12" t="s">
+        <v>293</v>
+      </c>
+      <c r="D72" s="13"/>
+      <c r="E72" s="13" t="s">
+        <v>294</v>
       </c>
       <c r="F72" s="3"/>
       <c r="G72" s="3"/>
@@ -4350,17 +4359,13 @@
       <c r="A73" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="B73" s="3" t="s">
-        <v>129</v>
-      </c>
+      <c r="B73" s="3"/>
       <c r="C73" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="D73" s="3" t="s">
-        <v>130</v>
-      </c>
+      <c r="D73" s="3"/>
       <c r="E73" s="3" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="F73" s="3"/>
       <c r="G73" s="3"/>
@@ -4392,16 +4397,16 @@
         <v>127</v>
       </c>
       <c r="B74" s="3" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="C74" s="1" t="s">
         <v>127</v>
       </c>
       <c r="D74" s="3" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="E74" s="3" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="F74" s="3"/>
       <c r="G74" s="3"/>
@@ -4433,16 +4438,16 @@
         <v>127</v>
       </c>
       <c r="B75" s="3" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="C75" s="1" t="s">
         <v>127</v>
       </c>
       <c r="D75" s="3" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="E75" s="3" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="F75" s="3"/>
       <c r="G75" s="3"/>
@@ -4470,20 +4475,20 @@
       <c r="AC75" s="3"/>
     </row>
     <row r="76" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A76" s="27" t="s">
+      <c r="A76" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="B76" s="28" t="s">
-        <v>313</v>
-      </c>
-      <c r="C76" s="27" t="s">
+      <c r="B76" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="C76" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="D76" s="28" t="s">
-        <v>313</v>
-      </c>
-      <c r="E76" s="28" t="s">
-        <v>314</v>
+      <c r="D76" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="E76" s="3" t="s">
+        <v>137</v>
       </c>
       <c r="F76" s="3"/>
       <c r="G76" s="3"/>
@@ -4511,20 +4516,20 @@
       <c r="AC76" s="3"/>
     </row>
     <row r="77" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A77" s="9" t="s">
+      <c r="A77" s="27" t="s">
         <v>127</v>
       </c>
-      <c r="B77" s="10" t="s">
-        <v>138</v>
-      </c>
-      <c r="C77" s="9" t="s">
+      <c r="B77" s="28" t="s">
+        <v>313</v>
+      </c>
+      <c r="C77" s="27" t="s">
         <v>127</v>
       </c>
-      <c r="D77" s="10" t="s">
-        <v>139</v>
-      </c>
-      <c r="E77" s="10" t="s">
-        <v>140</v>
+      <c r="D77" s="28" t="s">
+        <v>313</v>
+      </c>
+      <c r="E77" s="28" t="s">
+        <v>314</v>
       </c>
       <c r="F77" s="3"/>
       <c r="G77" s="3"/>
@@ -4556,16 +4561,16 @@
         <v>127</v>
       </c>
       <c r="B78" s="10" t="s">
-        <v>270</v>
+        <v>138</v>
       </c>
       <c r="C78" s="9" t="s">
         <v>127</v>
       </c>
       <c r="D78" s="10" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="E78" s="10" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="F78" s="3"/>
       <c r="G78" s="3"/>
@@ -4593,20 +4598,20 @@
       <c r="AC78" s="3"/>
     </row>
     <row r="79" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A79" s="12" t="s">
+      <c r="A79" s="9" t="s">
         <v>127</v>
       </c>
-      <c r="B79" s="13" t="s">
-        <v>295</v>
-      </c>
-      <c r="C79" s="12" t="s">
+      <c r="B79" s="10" t="s">
+        <v>270</v>
+      </c>
+      <c r="C79" s="9" t="s">
         <v>127</v>
       </c>
-      <c r="D79" s="13" t="s">
-        <v>296</v>
-      </c>
-      <c r="E79" s="13" t="s">
-        <v>297</v>
+      <c r="D79" s="10" t="s">
+        <v>141</v>
+      </c>
+      <c r="E79" s="10" t="s">
+        <v>142</v>
       </c>
       <c r="F79" s="3"/>
       <c r="G79" s="3"/>
@@ -4634,16 +4639,20 @@
       <c r="AC79" s="3"/>
     </row>
     <row r="80" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A80" s="9" t="s">
-        <v>143</v>
-      </c>
-      <c r="B80" s="10"/>
-      <c r="C80" s="9" t="s">
-        <v>143</v>
-      </c>
-      <c r="D80" s="10"/>
-      <c r="E80" s="3" t="s">
-        <v>144</v>
+      <c r="A80" s="12" t="s">
+        <v>127</v>
+      </c>
+      <c r="B80" s="13" t="s">
+        <v>295</v>
+      </c>
+      <c r="C80" s="12" t="s">
+        <v>127</v>
+      </c>
+      <c r="D80" s="13" t="s">
+        <v>296</v>
+      </c>
+      <c r="E80" s="13" t="s">
+        <v>297</v>
       </c>
       <c r="F80" s="3"/>
       <c r="G80" s="3"/>
@@ -4671,16 +4680,16 @@
       <c r="AC80" s="3"/>
     </row>
     <row r="81" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A81" s="1" t="s">
-        <v>145</v>
-      </c>
-      <c r="B81" s="3"/>
-      <c r="C81" s="1" t="s">
-        <v>145</v>
-      </c>
-      <c r="D81" s="3"/>
+      <c r="A81" s="9" t="s">
+        <v>143</v>
+      </c>
+      <c r="B81" s="10"/>
+      <c r="C81" s="9" t="s">
+        <v>143</v>
+      </c>
+      <c r="D81" s="10"/>
       <c r="E81" s="3" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="F81" s="3"/>
       <c r="G81" s="3"/>
@@ -4708,20 +4717,16 @@
       <c r="AC81" s="3"/>
     </row>
     <row r="82" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A82" s="12" t="s">
-        <v>219</v>
-      </c>
-      <c r="B82" s="13" t="s">
-        <v>298</v>
-      </c>
-      <c r="C82" s="12" t="s">
-        <v>219</v>
-      </c>
-      <c r="D82" s="13" t="s">
-        <v>298</v>
-      </c>
-      <c r="E82" s="13" t="s">
-        <v>299</v>
+      <c r="A82" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="B82" s="3"/>
+      <c r="C82" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="D82" s="3"/>
+      <c r="E82" s="3" t="s">
+        <v>146</v>
       </c>
       <c r="F82" s="3"/>
       <c r="G82" s="3"/>
@@ -4753,16 +4758,16 @@
         <v>219</v>
       </c>
       <c r="B83" s="13" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
       <c r="C83" s="12" t="s">
         <v>219</v>
       </c>
       <c r="D83" s="13" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
       <c r="E83" s="13" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
       <c r="F83" s="3"/>
       <c r="G83" s="3"/>
@@ -4794,16 +4799,16 @@
         <v>219</v>
       </c>
       <c r="B84" s="13" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="C84" s="12" t="s">
         <v>219</v>
       </c>
       <c r="D84" s="13" t="s">
-        <v>303</v>
+        <v>300</v>
       </c>
       <c r="E84" s="13" t="s">
-        <v>304</v>
+        <v>301</v>
       </c>
       <c r="F84" s="3"/>
       <c r="G84" s="3"/>
@@ -4831,20 +4836,20 @@
       <c r="AC84" s="3"/>
     </row>
     <row r="85" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A85" s="1" t="s">
-        <v>147</v>
-      </c>
-      <c r="B85" s="3" t="s">
-        <v>148</v>
-      </c>
-      <c r="C85" s="1" t="s">
-        <v>147</v>
-      </c>
-      <c r="D85" s="3" t="s">
-        <v>148</v>
-      </c>
-      <c r="E85" s="3" t="s">
-        <v>149</v>
+      <c r="A85" s="12" t="s">
+        <v>219</v>
+      </c>
+      <c r="B85" s="13" t="s">
+        <v>302</v>
+      </c>
+      <c r="C85" s="12" t="s">
+        <v>219</v>
+      </c>
+      <c r="D85" s="13" t="s">
+        <v>303</v>
+      </c>
+      <c r="E85" s="13" t="s">
+        <v>304</v>
       </c>
       <c r="F85" s="3"/>
       <c r="G85" s="3"/>
@@ -4872,20 +4877,20 @@
       <c r="AC85" s="3"/>
     </row>
     <row r="86" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A86" s="9" t="s">
+      <c r="A86" s="1" t="s">
         <v>147</v>
       </c>
-      <c r="B86" s="10" t="s">
-        <v>150</v>
-      </c>
-      <c r="C86" s="9" t="s">
+      <c r="B86" s="3" t="s">
+        <v>148</v>
+      </c>
+      <c r="C86" s="1" t="s">
         <v>147</v>
       </c>
-      <c r="D86" s="10" t="s">
-        <v>150</v>
-      </c>
-      <c r="E86" s="11" t="s">
-        <v>151</v>
+      <c r="D86" s="3" t="s">
+        <v>148</v>
+      </c>
+      <c r="E86" s="3" t="s">
+        <v>149</v>
       </c>
       <c r="F86" s="3"/>
       <c r="G86" s="3"/>
@@ -4917,16 +4922,16 @@
         <v>147</v>
       </c>
       <c r="B87" s="10" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="C87" s="9" t="s">
         <v>147</v>
       </c>
       <c r="D87" s="10" t="s">
-        <v>152</v>
-      </c>
-      <c r="E87" s="3" t="s">
-        <v>153</v>
+        <v>150</v>
+      </c>
+      <c r="E87" s="11" t="s">
+        <v>151</v>
       </c>
       <c r="F87" s="3"/>
       <c r="G87" s="3"/>
@@ -4954,20 +4959,20 @@
       <c r="AC87" s="3"/>
     </row>
     <row r="88" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A88" s="1" t="s">
+      <c r="A88" s="9" t="s">
         <v>147</v>
       </c>
-      <c r="B88" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="C88" s="1" t="s">
+      <c r="B88" s="10" t="s">
+        <v>152</v>
+      </c>
+      <c r="C88" s="9" t="s">
         <v>147</v>
       </c>
-      <c r="D88" s="3" t="s">
-        <v>25</v>
+      <c r="D88" s="10" t="s">
+        <v>152</v>
       </c>
       <c r="E88" s="3" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="F88" s="3"/>
       <c r="G88" s="3"/>
@@ -4999,16 +5004,16 @@
         <v>147</v>
       </c>
       <c r="B89" s="3" t="s">
-        <v>155</v>
+        <v>23</v>
       </c>
       <c r="C89" s="1" t="s">
         <v>147</v>
       </c>
       <c r="D89" s="3" t="s">
-        <v>156</v>
+        <v>25</v>
       </c>
       <c r="E89" s="3" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="F89" s="3"/>
       <c r="G89" s="3"/>
@@ -5036,20 +5041,20 @@
       <c r="AC89" s="3"/>
     </row>
     <row r="90" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A90" s="9" t="s">
+      <c r="A90" s="1" t="s">
         <v>147</v>
       </c>
-      <c r="B90" s="10" t="s">
-        <v>158</v>
-      </c>
-      <c r="C90" s="9" t="s">
+      <c r="B90" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="C90" s="1" t="s">
         <v>147</v>
       </c>
-      <c r="D90" s="10" t="s">
-        <v>159</v>
-      </c>
-      <c r="E90" s="11" t="s">
-        <v>160</v>
+      <c r="D90" s="3" t="s">
+        <v>156</v>
+      </c>
+      <c r="E90" s="3" t="s">
+        <v>157</v>
       </c>
       <c r="F90" s="3"/>
       <c r="G90" s="3"/>
@@ -5081,16 +5086,16 @@
         <v>147</v>
       </c>
       <c r="B91" s="10" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="C91" s="9" t="s">
         <v>147</v>
       </c>
       <c r="D91" s="10" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="E91" s="11" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="F91" s="3"/>
       <c r="G91" s="3"/>
@@ -5122,16 +5127,16 @@
         <v>147</v>
       </c>
       <c r="B92" s="10" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="C92" s="9" t="s">
         <v>147</v>
       </c>
       <c r="D92" s="10" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="E92" s="11" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="F92" s="3"/>
       <c r="G92" s="3"/>
@@ -5159,20 +5164,20 @@
       <c r="AC92" s="3"/>
     </row>
     <row r="93" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A93" s="1" t="s">
+      <c r="A93" s="9" t="s">
         <v>147</v>
       </c>
-      <c r="B93" s="3" t="s">
-        <v>165</v>
-      </c>
-      <c r="C93" s="1" t="s">
+      <c r="B93" s="10" t="s">
+        <v>163</v>
+      </c>
+      <c r="C93" s="9" t="s">
         <v>147</v>
       </c>
-      <c r="D93" s="3" t="s">
-        <v>165</v>
+      <c r="D93" s="10" t="s">
+        <v>163</v>
       </c>
       <c r="E93" s="11" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="F93" s="3"/>
       <c r="G93" s="3"/>
@@ -5200,20 +5205,20 @@
       <c r="AC93" s="3"/>
     </row>
     <row r="94" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A94" s="12" t="s">
+      <c r="A94" s="1" t="s">
         <v>147</v>
       </c>
-      <c r="B94" s="13" t="s">
-        <v>305</v>
-      </c>
-      <c r="C94" s="12" t="s">
+      <c r="B94" s="3" t="s">
+        <v>165</v>
+      </c>
+      <c r="C94" s="1" t="s">
         <v>147</v>
       </c>
-      <c r="D94" s="13" t="s">
-        <v>305</v>
-      </c>
-      <c r="E94" s="13" t="s">
-        <v>306</v>
+      <c r="D94" s="3" t="s">
+        <v>165</v>
+      </c>
+      <c r="E94" s="11" t="s">
+        <v>166</v>
       </c>
       <c r="F94" s="3"/>
       <c r="G94" s="3"/>
@@ -5241,20 +5246,20 @@
       <c r="AC94" s="3"/>
     </row>
     <row r="95" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A95" s="1" t="s">
+      <c r="A95" s="12" t="s">
         <v>147</v>
       </c>
-      <c r="B95" s="3" t="s">
-        <v>167</v>
-      </c>
-      <c r="C95" s="1" t="s">
+      <c r="B95" s="13" t="s">
+        <v>305</v>
+      </c>
+      <c r="C95" s="12" t="s">
         <v>147</v>
       </c>
-      <c r="D95" s="3" t="s">
-        <v>167</v>
-      </c>
-      <c r="E95" s="11" t="s">
-        <v>168</v>
+      <c r="D95" s="13" t="s">
+        <v>305</v>
+      </c>
+      <c r="E95" s="13" t="s">
+        <v>306</v>
       </c>
       <c r="F95" s="3"/>
       <c r="G95" s="3"/>
@@ -5286,16 +5291,16 @@
         <v>147</v>
       </c>
       <c r="B96" s="3" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="C96" s="1" t="s">
         <v>147</v>
       </c>
       <c r="D96" s="3" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="E96" s="11" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="F96" s="3"/>
       <c r="G96" s="3"/>
@@ -5327,16 +5332,16 @@
         <v>147</v>
       </c>
       <c r="B97" s="3" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="C97" s="1" t="s">
         <v>147</v>
       </c>
       <c r="D97" s="3" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="E97" s="11" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="F97" s="3"/>
       <c r="G97" s="3"/>
@@ -5364,20 +5369,20 @@
       <c r="AC97" s="3"/>
     </row>
     <row r="98" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A98" s="9" t="s">
+      <c r="A98" s="1" t="s">
         <v>147</v>
       </c>
-      <c r="B98" s="10" t="s">
-        <v>173</v>
-      </c>
-      <c r="C98" s="9" t="s">
+      <c r="B98" s="3" t="s">
+        <v>171</v>
+      </c>
+      <c r="C98" s="1" t="s">
         <v>147</v>
       </c>
-      <c r="D98" s="10" t="s">
-        <v>173</v>
+      <c r="D98" s="3" t="s">
+        <v>171</v>
       </c>
       <c r="E98" s="11" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="F98" s="3"/>
       <c r="G98" s="3"/>
@@ -5405,20 +5410,20 @@
       <c r="AC98" s="3"/>
     </row>
     <row r="99" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A99" s="12" t="s">
+      <c r="A99" s="9" t="s">
         <v>147</v>
       </c>
-      <c r="B99" s="13" t="s">
-        <v>307</v>
-      </c>
-      <c r="C99" s="12" t="s">
+      <c r="B99" s="10" t="s">
+        <v>173</v>
+      </c>
+      <c r="C99" s="9" t="s">
         <v>147</v>
       </c>
-      <c r="D99" s="13" t="s">
-        <v>307</v>
-      </c>
-      <c r="E99" s="13" t="s">
-        <v>308</v>
+      <c r="D99" s="10" t="s">
+        <v>173</v>
+      </c>
+      <c r="E99" s="11" t="s">
+        <v>174</v>
       </c>
       <c r="F99" s="3"/>
       <c r="G99" s="3"/>
@@ -5446,20 +5451,20 @@
       <c r="AC99" s="3"/>
     </row>
     <row r="100" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A100" s="9" t="s">
+      <c r="A100" s="12" t="s">
         <v>147</v>
       </c>
-      <c r="B100" s="23" t="s">
-        <v>175</v>
-      </c>
-      <c r="C100" s="9" t="s">
+      <c r="B100" s="13" t="s">
+        <v>307</v>
+      </c>
+      <c r="C100" s="12" t="s">
         <v>147</v>
       </c>
-      <c r="D100" s="23" t="s">
-        <v>176</v>
-      </c>
-      <c r="E100" s="24" t="s">
-        <v>177</v>
+      <c r="D100" s="13" t="s">
+        <v>307</v>
+      </c>
+      <c r="E100" s="13" t="s">
+        <v>308</v>
       </c>
       <c r="F100" s="3"/>
       <c r="G100" s="3"/>
@@ -5491,16 +5496,16 @@
         <v>147</v>
       </c>
       <c r="B101" s="23" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="C101" s="9" t="s">
         <v>147</v>
       </c>
       <c r="D101" s="23" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="E101" s="24" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="F101" s="3"/>
       <c r="G101" s="3"/>
@@ -5528,20 +5533,20 @@
       <c r="AC101" s="3"/>
     </row>
     <row r="102" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A102" s="1" t="s">
+      <c r="A102" s="9" t="s">
         <v>147</v>
       </c>
-      <c r="B102" s="7" t="s">
-        <v>180</v>
-      </c>
-      <c r="C102" s="1" t="s">
+      <c r="B102" s="23" t="s">
+        <v>178</v>
+      </c>
+      <c r="C102" s="9" t="s">
         <v>147</v>
       </c>
-      <c r="D102" s="7" t="s">
-        <v>181</v>
-      </c>
-      <c r="E102" s="18" t="s">
-        <v>182</v>
+      <c r="D102" s="23" t="s">
+        <v>178</v>
+      </c>
+      <c r="E102" s="24" t="s">
+        <v>179</v>
       </c>
       <c r="F102" s="3"/>
       <c r="G102" s="3"/>
@@ -5569,20 +5574,20 @@
       <c r="AC102" s="3"/>
     </row>
     <row r="103" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A103" s="25" t="s">
+      <c r="A103" s="1" t="s">
         <v>147</v>
       </c>
-      <c r="B103" s="26" t="s">
-        <v>183</v>
-      </c>
-      <c r="C103" s="25" t="s">
+      <c r="B103" s="7" t="s">
+        <v>180</v>
+      </c>
+      <c r="C103" s="1" t="s">
         <v>147</v>
       </c>
-      <c r="D103" s="26" t="s">
-        <v>184</v>
-      </c>
-      <c r="E103" s="11" t="s">
-        <v>185</v>
+      <c r="D103" s="7" t="s">
+        <v>181</v>
+      </c>
+      <c r="E103" s="18" t="s">
+        <v>182</v>
       </c>
       <c r="F103" s="3"/>
       <c r="G103" s="3"/>
@@ -5610,20 +5615,20 @@
       <c r="AC103" s="3"/>
     </row>
     <row r="104" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A104" s="9" t="s">
+      <c r="A104" s="25" t="s">
         <v>147</v>
       </c>
-      <c r="B104" s="10" t="s">
-        <v>186</v>
-      </c>
-      <c r="C104" s="9" t="s">
+      <c r="B104" s="26" t="s">
+        <v>183</v>
+      </c>
+      <c r="C104" s="25" t="s">
         <v>147</v>
       </c>
-      <c r="D104" s="10" t="s">
-        <v>187</v>
+      <c r="D104" s="26" t="s">
+        <v>184</v>
       </c>
       <c r="E104" s="11" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
       <c r="F104" s="3"/>
       <c r="G104" s="3"/>
@@ -5651,20 +5656,20 @@
       <c r="AC104" s="3"/>
     </row>
     <row r="105" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A105" s="1" t="s">
+      <c r="A105" s="9" t="s">
         <v>147</v>
       </c>
-      <c r="B105" s="3" t="s">
-        <v>189</v>
-      </c>
-      <c r="C105" s="1" t="s">
+      <c r="B105" s="10" t="s">
+        <v>186</v>
+      </c>
+      <c r="C105" s="9" t="s">
         <v>147</v>
       </c>
-      <c r="D105" s="3" t="s">
-        <v>190</v>
+      <c r="D105" s="10" t="s">
+        <v>187</v>
       </c>
       <c r="E105" s="11" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="F105" s="3"/>
       <c r="G105" s="3"/>
@@ -5696,16 +5701,16 @@
         <v>147</v>
       </c>
       <c r="B106" s="3" t="s">
-        <v>192</v>
+        <v>189</v>
       </c>
       <c r="C106" s="1" t="s">
         <v>147</v>
       </c>
       <c r="D106" s="3" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="E106" s="11" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="F106" s="3"/>
       <c r="G106" s="3"/>
@@ -5734,19 +5739,19 @@
     </row>
     <row r="107" spans="1:29" ht="15.75" customHeight="1">
       <c r="A107" s="1" t="s">
-        <v>194</v>
+        <v>147</v>
       </c>
       <c r="B107" s="3" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="C107" s="1" t="s">
-        <v>194</v>
+        <v>147</v>
       </c>
       <c r="D107" s="3" t="s">
-        <v>196</v>
+        <v>192</v>
       </c>
       <c r="E107" s="11" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
       <c r="F107" s="3"/>
       <c r="G107" s="3"/>
@@ -5775,15 +5780,19 @@
     </row>
     <row r="108" spans="1:29" ht="15.75" customHeight="1">
       <c r="A108" s="1" t="s">
-        <v>198</v>
-      </c>
-      <c r="B108" s="3"/>
+        <v>194</v>
+      </c>
+      <c r="B108" s="3" t="s">
+        <v>195</v>
+      </c>
       <c r="C108" s="1" t="s">
-        <v>199</v>
-      </c>
-      <c r="D108" s="3"/>
+        <v>194</v>
+      </c>
+      <c r="D108" s="3" t="s">
+        <v>196</v>
+      </c>
       <c r="E108" s="11" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="F108" s="3"/>
       <c r="G108" s="3"/>
@@ -5811,16 +5820,16 @@
       <c r="AC108" s="3"/>
     </row>
     <row r="109" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A109" s="25" t="s">
-        <v>201</v>
-      </c>
-      <c r="B109" s="26"/>
-      <c r="C109" s="25" t="s">
-        <v>201</v>
-      </c>
-      <c r="D109" s="26"/>
-      <c r="E109" s="3" t="s">
-        <v>202</v>
+      <c r="A109" s="1" t="s">
+        <v>198</v>
+      </c>
+      <c r="B109" s="3"/>
+      <c r="C109" s="1" t="s">
+        <v>199</v>
+      </c>
+      <c r="D109" s="3"/>
+      <c r="E109" s="11" t="s">
+        <v>200</v>
       </c>
       <c r="F109" s="3"/>
       <c r="G109" s="3"/>
@@ -5848,16 +5857,16 @@
       <c r="AC109" s="3"/>
     </row>
     <row r="110" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A110" s="9" t="s">
-        <v>203</v>
-      </c>
-      <c r="B110" s="10"/>
-      <c r="C110" s="9" t="s">
-        <v>203</v>
-      </c>
-      <c r="D110" s="10"/>
-      <c r="E110" s="11" t="s">
-        <v>204</v>
+      <c r="A110" s="25" t="s">
+        <v>201</v>
+      </c>
+      <c r="B110" s="26"/>
+      <c r="C110" s="25" t="s">
+        <v>201</v>
+      </c>
+      <c r="D110" s="26"/>
+      <c r="E110" s="3" t="s">
+        <v>202</v>
       </c>
       <c r="F110" s="3"/>
       <c r="G110" s="3"/>
@@ -5885,16 +5894,16 @@
       <c r="AC110" s="3"/>
     </row>
     <row r="111" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A111" s="1" t="s">
-        <v>205</v>
-      </c>
-      <c r="B111" s="3"/>
-      <c r="C111" s="1" t="s">
-        <v>205</v>
-      </c>
-      <c r="D111" s="3"/>
-      <c r="E111" s="3" t="s">
-        <v>206</v>
+      <c r="A111" s="9" t="s">
+        <v>203</v>
+      </c>
+      <c r="B111" s="10"/>
+      <c r="C111" s="9" t="s">
+        <v>203</v>
+      </c>
+      <c r="D111" s="10"/>
+      <c r="E111" s="11" t="s">
+        <v>204</v>
       </c>
       <c r="F111" s="3"/>
       <c r="G111" s="3"/>
@@ -5923,19 +5932,15 @@
     </row>
     <row r="112" spans="1:29" ht="15.75" customHeight="1">
       <c r="A112" s="1" t="s">
-        <v>207</v>
-      </c>
-      <c r="B112" s="3" t="s">
-        <v>167</v>
-      </c>
+        <v>205</v>
+      </c>
+      <c r="B112" s="3"/>
       <c r="C112" s="1" t="s">
-        <v>208</v>
-      </c>
-      <c r="D112" s="3" t="s">
-        <v>167</v>
-      </c>
+        <v>205</v>
+      </c>
+      <c r="D112" s="3"/>
       <c r="E112" s="3" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="F112" s="3"/>
       <c r="G112" s="3"/>
@@ -5967,16 +5972,16 @@
         <v>207</v>
       </c>
       <c r="B113" s="3" t="s">
-        <v>210</v>
+        <v>167</v>
       </c>
       <c r="C113" s="1" t="s">
         <v>208</v>
       </c>
       <c r="D113" s="3" t="s">
-        <v>210</v>
+        <v>167</v>
       </c>
       <c r="E113" s="3" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="F113" s="3"/>
       <c r="G113" s="3"/>
@@ -6004,20 +6009,20 @@
       <c r="AC113" s="3"/>
     </row>
     <row r="114" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A114" s="9" t="s">
+      <c r="A114" s="1" t="s">
         <v>207</v>
       </c>
-      <c r="B114" s="10" t="s">
-        <v>165</v>
+      <c r="B114" s="3" t="s">
+        <v>210</v>
       </c>
       <c r="C114" s="1" t="s">
         <v>208</v>
       </c>
-      <c r="D114" s="10" t="s">
-        <v>165</v>
-      </c>
-      <c r="E114" s="10" t="s">
-        <v>212</v>
+      <c r="D114" s="3" t="s">
+        <v>210</v>
+      </c>
+      <c r="E114" s="3" t="s">
+        <v>211</v>
       </c>
       <c r="F114" s="3"/>
       <c r="G114" s="3"/>
@@ -6045,20 +6050,20 @@
       <c r="AC114" s="3"/>
     </row>
     <row r="115" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A115" s="1" t="s">
-        <v>213</v>
-      </c>
-      <c r="B115" s="3" t="s">
-        <v>214</v>
+      <c r="A115" s="9" t="s">
+        <v>207</v>
+      </c>
+      <c r="B115" s="10" t="s">
+        <v>165</v>
       </c>
       <c r="C115" s="1" t="s">
-        <v>213</v>
-      </c>
-      <c r="D115" s="3" t="s">
-        <v>214</v>
-      </c>
-      <c r="E115" s="3" t="s">
-        <v>215</v>
+        <v>208</v>
+      </c>
+      <c r="D115" s="10" t="s">
+        <v>165</v>
+      </c>
+      <c r="E115" s="10" t="s">
+        <v>212</v>
       </c>
       <c r="F115" s="3"/>
       <c r="G115" s="3"/>
@@ -6086,20 +6091,20 @@
       <c r="AC115" s="3"/>
     </row>
     <row r="116" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A116" s="3" t="s">
+      <c r="A116" s="1" t="s">
         <v>213</v>
       </c>
       <c r="B116" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="C116" s="3" t="s">
+        <v>214</v>
+      </c>
+      <c r="C116" s="1" t="s">
         <v>213</v>
       </c>
       <c r="D116" s="3" t="s">
-        <v>57</v>
+        <v>214</v>
       </c>
       <c r="E116" s="3" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="F116" s="3"/>
       <c r="G116" s="3"/>
@@ -6131,16 +6136,16 @@
         <v>213</v>
       </c>
       <c r="B117" s="3" t="s">
-        <v>217</v>
+        <v>57</v>
       </c>
       <c r="C117" s="3" t="s">
         <v>213</v>
       </c>
       <c r="D117" s="3" t="s">
-        <v>217</v>
+        <v>57</v>
       </c>
       <c r="E117" s="3" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="F117" s="3"/>
       <c r="G117" s="3"/>
@@ -6168,20 +6173,20 @@
       <c r="AC117" s="3"/>
     </row>
     <row r="118" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A118" s="1" t="s">
+      <c r="A118" s="3" t="s">
         <v>213</v>
       </c>
       <c r="B118" s="3" t="s">
-        <v>219</v>
-      </c>
-      <c r="C118" s="1" t="s">
+        <v>217</v>
+      </c>
+      <c r="C118" s="3" t="s">
         <v>213</v>
       </c>
       <c r="D118" s="3" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="E118" s="3" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="F118" s="3"/>
       <c r="G118" s="3"/>
@@ -6209,16 +6214,20 @@
       <c r="AC118" s="3"/>
     </row>
     <row r="119" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A119" s="9" t="s">
-        <v>221</v>
-      </c>
-      <c r="B119" s="10"/>
-      <c r="C119" s="9" t="s">
-        <v>221</v>
-      </c>
-      <c r="D119" s="10"/>
-      <c r="E119" s="11" t="s">
-        <v>222</v>
+      <c r="A119" s="1" t="s">
+        <v>213</v>
+      </c>
+      <c r="B119" s="3" t="s">
+        <v>219</v>
+      </c>
+      <c r="C119" s="1" t="s">
+        <v>213</v>
+      </c>
+      <c r="D119" s="3" t="s">
+        <v>219</v>
+      </c>
+      <c r="E119" s="3" t="s">
+        <v>220</v>
       </c>
       <c r="F119" s="3"/>
       <c r="G119" s="3"/>
@@ -6246,20 +6255,16 @@
       <c r="AC119" s="3"/>
     </row>
     <row r="120" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A120" s="30" t="s">
-        <v>320</v>
-      </c>
-      <c r="B120" s="31" t="s">
-        <v>321</v>
-      </c>
-      <c r="C120" s="30" t="s">
-        <v>322</v>
-      </c>
-      <c r="D120" s="31" t="s">
-        <v>321</v>
-      </c>
-      <c r="E120" s="32" t="s">
-        <v>323</v>
+      <c r="A120" s="9" t="s">
+        <v>221</v>
+      </c>
+      <c r="B120" s="10"/>
+      <c r="C120" s="9" t="s">
+        <v>221</v>
+      </c>
+      <c r="D120" s="10"/>
+      <c r="E120" s="11" t="s">
+        <v>222</v>
       </c>
       <c r="F120" s="3"/>
       <c r="G120" s="3"/>
@@ -6291,16 +6296,16 @@
         <v>320</v>
       </c>
       <c r="B121" s="31" t="s">
-        <v>341</v>
+        <v>321</v>
       </c>
       <c r="C121" s="30" t="s">
         <v>322</v>
       </c>
       <c r="D121" s="31" t="s">
-        <v>341</v>
+        <v>321</v>
       </c>
       <c r="E121" s="32" t="s">
-        <v>342</v>
+        <v>323</v>
       </c>
       <c r="F121" s="3"/>
       <c r="G121" s="3"/>
@@ -6332,16 +6337,16 @@
         <v>320</v>
       </c>
       <c r="B122" s="31" t="s">
-        <v>324</v>
+        <v>341</v>
       </c>
       <c r="C122" s="30" t="s">
         <v>322</v>
       </c>
       <c r="D122" s="31" t="s">
-        <v>324</v>
+        <v>341</v>
       </c>
       <c r="E122" s="32" t="s">
-        <v>325</v>
+        <v>342</v>
       </c>
       <c r="F122" s="3"/>
       <c r="G122" s="3"/>
@@ -6369,16 +6374,20 @@
       <c r="AC122" s="3"/>
     </row>
     <row r="123" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A123" s="12" t="s">
-        <v>309</v>
-      </c>
-      <c r="B123" s="13"/>
-      <c r="C123" s="12" t="s">
-        <v>309</v>
-      </c>
-      <c r="D123" s="13"/>
-      <c r="E123" s="13" t="s">
-        <v>310</v>
+      <c r="A123" s="30" t="s">
+        <v>320</v>
+      </c>
+      <c r="B123" s="31" t="s">
+        <v>324</v>
+      </c>
+      <c r="C123" s="30" t="s">
+        <v>322</v>
+      </c>
+      <c r="D123" s="31" t="s">
+        <v>324</v>
+      </c>
+      <c r="E123" s="32" t="s">
+        <v>325</v>
       </c>
       <c r="F123" s="3"/>
       <c r="G123" s="3"/>
@@ -6406,16 +6415,16 @@
       <c r="AC123" s="3"/>
     </row>
     <row r="124" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A124" s="1" t="s">
-        <v>223</v>
-      </c>
-      <c r="B124" s="3"/>
-      <c r="C124" s="1" t="s">
-        <v>223</v>
-      </c>
-      <c r="D124" s="3"/>
-      <c r="E124" s="3" t="s">
-        <v>224</v>
+      <c r="A124" s="12" t="s">
+        <v>309</v>
+      </c>
+      <c r="B124" s="13"/>
+      <c r="C124" s="12" t="s">
+        <v>309</v>
+      </c>
+      <c r="D124" s="13"/>
+      <c r="E124" s="13" t="s">
+        <v>310</v>
       </c>
       <c r="F124" s="3"/>
       <c r="G124" s="3"/>
@@ -6443,20 +6452,16 @@
       <c r="AC124" s="3"/>
     </row>
     <row r="125" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A125" s="3" t="s">
+      <c r="A125" s="1" t="s">
         <v>223</v>
       </c>
-      <c r="B125" s="3" t="s">
-        <v>225</v>
-      </c>
-      <c r="C125" s="3" t="s">
+      <c r="B125" s="3"/>
+      <c r="C125" s="1" t="s">
         <v>223</v>
       </c>
-      <c r="D125" s="3" t="s">
-        <v>226</v>
-      </c>
+      <c r="D125" s="3"/>
       <c r="E125" s="3" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="F125" s="3"/>
       <c r="G125" s="3"/>
@@ -6484,20 +6489,20 @@
       <c r="AC125" s="3"/>
     </row>
     <row r="126" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A126" s="1" t="s">
+      <c r="A126" s="3" t="s">
         <v>223</v>
       </c>
       <c r="B126" s="3" t="s">
-        <v>228</v>
-      </c>
-      <c r="C126" s="1" t="s">
+        <v>225</v>
+      </c>
+      <c r="C126" s="3" t="s">
         <v>223</v>
       </c>
       <c r="D126" s="3" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="E126" s="3" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="F126" s="3"/>
       <c r="G126" s="3"/>
@@ -6525,16 +6530,20 @@
       <c r="AC126" s="3"/>
     </row>
     <row r="127" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A127" s="9" t="s">
-        <v>230</v>
-      </c>
-      <c r="B127" s="10"/>
-      <c r="C127" s="9" t="s">
-        <v>230</v>
-      </c>
-      <c r="D127" s="10"/>
+      <c r="A127" s="1" t="s">
+        <v>223</v>
+      </c>
+      <c r="B127" s="3" t="s">
+        <v>228</v>
+      </c>
+      <c r="C127" s="1" t="s">
+        <v>223</v>
+      </c>
+      <c r="D127" s="3" t="s">
+        <v>228</v>
+      </c>
       <c r="E127" s="3" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="F127" s="3"/>
       <c r="G127" s="3"/>
@@ -6562,16 +6571,16 @@
       <c r="AC127" s="3"/>
     </row>
     <row r="128" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A128" s="1" t="s">
-        <v>210</v>
-      </c>
-      <c r="B128" s="3"/>
-      <c r="C128" s="1" t="s">
-        <v>210</v>
-      </c>
-      <c r="D128" s="3"/>
+      <c r="A128" s="9" t="s">
+        <v>230</v>
+      </c>
+      <c r="B128" s="10"/>
+      <c r="C128" s="9" t="s">
+        <v>230</v>
+      </c>
+      <c r="D128" s="10"/>
       <c r="E128" s="3" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="F128" s="3"/>
       <c r="G128" s="3"/>
@@ -6602,17 +6611,13 @@
       <c r="A129" s="1" t="s">
         <v>210</v>
       </c>
-      <c r="B129" s="3" t="s">
-        <v>233</v>
-      </c>
+      <c r="B129" s="3"/>
       <c r="C129" s="1" t="s">
         <v>210</v>
       </c>
-      <c r="D129" s="3" t="s">
-        <v>234</v>
-      </c>
+      <c r="D129" s="3"/>
       <c r="E129" s="3" t="s">
-        <v>235</v>
+        <v>232</v>
       </c>
       <c r="F129" s="3"/>
       <c r="G129" s="3"/>
@@ -6644,16 +6649,16 @@
         <v>210</v>
       </c>
       <c r="B130" s="3" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="C130" s="1" t="s">
         <v>210</v>
       </c>
       <c r="D130" s="3" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="E130" s="3" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="F130" s="3"/>
       <c r="G130" s="3"/>
@@ -6685,16 +6690,16 @@
         <v>210</v>
       </c>
       <c r="B131" s="3" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="C131" s="1" t="s">
         <v>210</v>
       </c>
       <c r="D131" s="3" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="E131" s="3" t="s">
-        <v>240</v>
+        <v>237</v>
       </c>
       <c r="F131" s="3"/>
       <c r="G131" s="3"/>
@@ -6726,16 +6731,16 @@
         <v>210</v>
       </c>
       <c r="B132" s="3" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="C132" s="1" t="s">
         <v>210</v>
       </c>
       <c r="D132" s="3" t="s">
-        <v>242</v>
+        <v>239</v>
       </c>
       <c r="E132" s="3" t="s">
-        <v>243</v>
+        <v>240</v>
       </c>
       <c r="F132" s="3"/>
       <c r="G132" s="3"/>
@@ -6767,16 +6772,16 @@
         <v>210</v>
       </c>
       <c r="B133" s="3" t="s">
-        <v>244</v>
+        <v>241</v>
       </c>
       <c r="C133" s="1" t="s">
         <v>210</v>
       </c>
       <c r="D133" s="3" t="s">
-        <v>245</v>
+        <v>242</v>
       </c>
       <c r="E133" s="3" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="F133" s="3"/>
       <c r="G133" s="3"/>
@@ -6808,16 +6813,16 @@
         <v>210</v>
       </c>
       <c r="B134" s="3" t="s">
-        <v>247</v>
+        <v>244</v>
       </c>
       <c r="C134" s="1" t="s">
         <v>210</v>
       </c>
       <c r="D134" s="3" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
       <c r="E134" s="3" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="F134" s="3"/>
       <c r="G134" s="3"/>
@@ -6849,16 +6854,16 @@
         <v>210</v>
       </c>
       <c r="B135" s="3" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="C135" s="1" t="s">
         <v>210</v>
       </c>
       <c r="D135" s="3" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="E135" s="3" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="F135" s="3"/>
       <c r="G135" s="3"/>
@@ -6890,16 +6895,16 @@
         <v>210</v>
       </c>
       <c r="B136" s="3" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="C136" s="1" t="s">
         <v>210</v>
       </c>
       <c r="D136" s="3" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="E136" s="3" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="F136" s="3"/>
       <c r="G136" s="3"/>
@@ -6931,16 +6936,16 @@
         <v>210</v>
       </c>
       <c r="B137" s="3" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="C137" s="1" t="s">
         <v>210</v>
       </c>
       <c r="D137" s="3" t="s">
-        <v>255</v>
+        <v>252</v>
       </c>
       <c r="E137" s="3" t="s">
-        <v>256</v>
+        <v>253</v>
       </c>
       <c r="F137" s="3"/>
       <c r="G137" s="3"/>
@@ -6972,16 +6977,16 @@
         <v>210</v>
       </c>
       <c r="B138" s="3" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
       <c r="C138" s="1" t="s">
         <v>210</v>
       </c>
       <c r="D138" s="3" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="E138" s="3" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="F138" s="3"/>
       <c r="G138" s="3"/>
@@ -7013,16 +7018,16 @@
         <v>210</v>
       </c>
       <c r="B139" s="3" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="C139" s="1" t="s">
         <v>210</v>
       </c>
       <c r="D139" s="3" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="E139" s="3" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="F139" s="3"/>
       <c r="G139" s="3"/>
@@ -7054,16 +7059,16 @@
         <v>210</v>
       </c>
       <c r="B140" s="3" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="C140" s="1" t="s">
         <v>210</v>
       </c>
       <c r="D140" s="3" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="E140" s="3" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="F140" s="3"/>
       <c r="G140" s="3"/>
@@ -7091,16 +7096,20 @@
       <c r="AC140" s="3"/>
     </row>
     <row r="141" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A141" s="25" t="s">
-        <v>311</v>
-      </c>
-      <c r="B141" s="26"/>
-      <c r="C141" s="25" t="s">
-        <v>311</v>
-      </c>
-      <c r="D141" s="26"/>
+      <c r="A141" s="1" t="s">
+        <v>210</v>
+      </c>
+      <c r="B141" s="3" t="s">
+        <v>261</v>
+      </c>
+      <c r="C141" s="1" t="s">
+        <v>210</v>
+      </c>
+      <c r="D141" s="3" t="s">
+        <v>261</v>
+      </c>
       <c r="E141" s="3" t="s">
-        <v>312</v>
+        <v>262</v>
       </c>
       <c r="F141" s="3"/>
       <c r="G141" s="3"/>
@@ -7128,16 +7137,16 @@
       <c r="AC141" s="3"/>
     </row>
     <row r="142" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A142" s="9" t="s">
-        <v>263</v>
-      </c>
-      <c r="B142" s="10"/>
-      <c r="C142" s="9" t="s">
-        <v>263</v>
-      </c>
-      <c r="D142" s="10"/>
+      <c r="A142" s="25" t="s">
+        <v>311</v>
+      </c>
+      <c r="B142" s="26"/>
+      <c r="C142" s="25" t="s">
+        <v>311</v>
+      </c>
+      <c r="D142" s="26"/>
       <c r="E142" s="3" t="s">
-        <v>264</v>
+        <v>312</v>
       </c>
       <c r="F142" s="3"/>
       <c r="G142" s="3"/>
@@ -7165,16 +7174,16 @@
       <c r="AC142" s="3"/>
     </row>
     <row r="143" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A143" s="1" t="s">
-        <v>265</v>
-      </c>
-      <c r="B143" s="3"/>
-      <c r="C143" s="1" t="s">
-        <v>265</v>
-      </c>
-      <c r="D143" s="3"/>
+      <c r="A143" s="9" t="s">
+        <v>263</v>
+      </c>
+      <c r="B143" s="10"/>
+      <c r="C143" s="9" t="s">
+        <v>263</v>
+      </c>
+      <c r="D143" s="10"/>
       <c r="E143" s="3" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="F143" s="3"/>
       <c r="G143" s="3"/>
@@ -7203,15 +7212,15 @@
     </row>
     <row r="144" spans="1:29" ht="15.75" customHeight="1">
       <c r="A144" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="B144" s="3"/>
       <c r="C144" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="D144" s="3"/>
       <c r="E144" s="3" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="F144" s="3"/>
       <c r="G144" s="3"/>
@@ -7238,54 +7247,54 @@
       <c r="AB144" s="3"/>
       <c r="AC144" s="3"/>
     </row>
-    <row r="145" spans="1:29" s="29" customFormat="1" ht="15.75" customHeight="1">
-      <c r="A145" s="28" t="s">
+    <row r="145" spans="1:29" ht="15.75" customHeight="1">
+      <c r="A145" s="1" t="s">
+        <v>267</v>
+      </c>
+      <c r="B145" s="3"/>
+      <c r="C145" s="1" t="s">
+        <v>267</v>
+      </c>
+      <c r="D145" s="3"/>
+      <c r="E145" s="3" t="s">
+        <v>268</v>
+      </c>
+      <c r="F145" s="3"/>
+      <c r="G145" s="3"/>
+      <c r="H145" s="3"/>
+      <c r="I145" s="3"/>
+      <c r="J145" s="3"/>
+      <c r="K145" s="3"/>
+      <c r="L145" s="3"/>
+      <c r="M145" s="3"/>
+      <c r="N145" s="3"/>
+      <c r="O145" s="3"/>
+      <c r="P145" s="3"/>
+      <c r="Q145" s="3"/>
+      <c r="R145" s="3"/>
+      <c r="S145" s="3"/>
+      <c r="T145" s="3"/>
+      <c r="U145" s="3"/>
+      <c r="V145" s="3"/>
+      <c r="W145" s="3"/>
+      <c r="X145" s="3"/>
+      <c r="Y145" s="3"/>
+      <c r="Z145" s="3"/>
+      <c r="AA145" s="3"/>
+      <c r="AB145" s="3"/>
+      <c r="AC145" s="3"/>
+    </row>
+    <row r="146" spans="1:29" s="29" customFormat="1" ht="15.75" customHeight="1">
+      <c r="A146" s="28" t="s">
         <v>315</v>
-      </c>
-      <c r="B145" s="28"/>
-      <c r="C145" s="28" t="s">
-        <v>316</v>
-      </c>
-      <c r="D145" s="28"/>
-      <c r="E145" s="28" t="s">
-        <v>317</v>
-      </c>
-      <c r="F145" s="28"/>
-      <c r="G145" s="28"/>
-      <c r="H145" s="28"/>
-      <c r="I145" s="28"/>
-      <c r="J145" s="28"/>
-      <c r="K145" s="28"/>
-      <c r="L145" s="28"/>
-      <c r="M145" s="28"/>
-      <c r="N145" s="28"/>
-      <c r="O145" s="28"/>
-      <c r="P145" s="28"/>
-      <c r="Q145" s="28"/>
-      <c r="R145" s="28"/>
-      <c r="S145" s="28"/>
-      <c r="T145" s="28"/>
-      <c r="U145" s="28"/>
-      <c r="V145" s="28"/>
-      <c r="W145" s="28"/>
-      <c r="X145" s="28"/>
-      <c r="Y145" s="28"/>
-      <c r="Z145" s="28"/>
-      <c r="AA145" s="28"/>
-      <c r="AB145" s="28"/>
-      <c r="AC145" s="28"/>
-    </row>
-    <row r="146" spans="1:29" s="29" customFormat="1" ht="15.75" customHeight="1">
-      <c r="A146" s="27" t="s">
-        <v>318</v>
       </c>
       <c r="B146" s="28"/>
       <c r="C146" s="28" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
       <c r="D146" s="28"/>
       <c r="E146" s="28" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
       <c r="F146" s="28"/>
       <c r="G146" s="28"/>
@@ -7312,39 +7321,45 @@
       <c r="AB146" s="28"/>
       <c r="AC146" s="28"/>
     </row>
-    <row r="147" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A147" s="3"/>
-      <c r="B147" s="3"/>
-      <c r="C147" s="3"/>
-      <c r="D147" s="3"/>
-      <c r="E147" s="3"/>
-      <c r="F147" s="3"/>
-      <c r="G147" s="3"/>
-      <c r="H147" s="3"/>
-      <c r="I147" s="3"/>
-      <c r="J147" s="3"/>
-      <c r="K147" s="3"/>
-      <c r="L147" s="3"/>
-      <c r="M147" s="3"/>
-      <c r="N147" s="3"/>
-      <c r="O147" s="3"/>
-      <c r="P147" s="3"/>
-      <c r="Q147" s="3"/>
-      <c r="R147" s="3"/>
-      <c r="S147" s="3"/>
-      <c r="T147" s="3"/>
-      <c r="U147" s="3"/>
-      <c r="V147" s="3"/>
-      <c r="W147" s="3"/>
-      <c r="X147" s="3"/>
-      <c r="Y147" s="3"/>
-      <c r="Z147" s="3"/>
-      <c r="AA147" s="3"/>
-      <c r="AB147" s="3"/>
-      <c r="AC147" s="3"/>
+    <row r="147" spans="1:29" s="29" customFormat="1" ht="15.75" customHeight="1">
+      <c r="A147" s="27" t="s">
+        <v>318</v>
+      </c>
+      <c r="B147" s="28"/>
+      <c r="C147" s="28" t="s">
+        <v>318</v>
+      </c>
+      <c r="D147" s="28"/>
+      <c r="E147" s="28" t="s">
+        <v>319</v>
+      </c>
+      <c r="F147" s="28"/>
+      <c r="G147" s="28"/>
+      <c r="H147" s="28"/>
+      <c r="I147" s="28"/>
+      <c r="J147" s="28"/>
+      <c r="K147" s="28"/>
+      <c r="L147" s="28"/>
+      <c r="M147" s="28"/>
+      <c r="N147" s="28"/>
+      <c r="O147" s="28"/>
+      <c r="P147" s="28"/>
+      <c r="Q147" s="28"/>
+      <c r="R147" s="28"/>
+      <c r="S147" s="28"/>
+      <c r="T147" s="28"/>
+      <c r="U147" s="28"/>
+      <c r="V147" s="28"/>
+      <c r="W147" s="28"/>
+      <c r="X147" s="28"/>
+      <c r="Y147" s="28"/>
+      <c r="Z147" s="28"/>
+      <c r="AA147" s="28"/>
+      <c r="AB147" s="28"/>
+      <c r="AC147" s="28"/>
     </row>
     <row r="148" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A148" s="1"/>
+      <c r="A148" s="3"/>
       <c r="B148" s="3"/>
       <c r="C148" s="3"/>
       <c r="D148" s="3"/>
@@ -7375,7 +7390,7 @@
       <c r="AC148" s="3"/>
     </row>
     <row r="149" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A149" s="3"/>
+      <c r="A149" s="1"/>
       <c r="B149" s="3"/>
       <c r="C149" s="3"/>
       <c r="D149" s="3"/>
@@ -35770,6 +35785,37 @@
       <c r="AB1064" s="3"/>
       <c r="AC1064" s="3"/>
     </row>
+    <row r="1065" spans="1:29" ht="15.75" customHeight="1">
+      <c r="A1065" s="3"/>
+      <c r="B1065" s="3"/>
+      <c r="C1065" s="3"/>
+      <c r="D1065" s="3"/>
+      <c r="E1065" s="3"/>
+      <c r="F1065" s="3"/>
+      <c r="G1065" s="3"/>
+      <c r="H1065" s="3"/>
+      <c r="I1065" s="3"/>
+      <c r="J1065" s="3"/>
+      <c r="K1065" s="3"/>
+      <c r="L1065" s="3"/>
+      <c r="M1065" s="3"/>
+      <c r="N1065" s="3"/>
+      <c r="O1065" s="3"/>
+      <c r="P1065" s="3"/>
+      <c r="Q1065" s="3"/>
+      <c r="R1065" s="3"/>
+      <c r="S1065" s="3"/>
+      <c r="T1065" s="3"/>
+      <c r="U1065" s="3"/>
+      <c r="V1065" s="3"/>
+      <c r="W1065" s="3"/>
+      <c r="X1065" s="3"/>
+      <c r="Y1065" s="3"/>
+      <c r="Z1065" s="3"/>
+      <c r="AA1065" s="3"/>
+      <c r="AB1065" s="3"/>
+      <c r="AC1065" s="3"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>

</xml_diff>